<commit_message>
Marca com asterisco os destinos com informação incompleta
Na aba 'Por país', o nome do destino recebe '* ' quando qualquer coluna
da linha contém informação a confirmar. Nota explicativa no Leia-me.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FBX8vzapzZkv77FqLGHwh3
</commit_message>
<xml_diff>
--- a/docs/Guia_Documentacao_Viagem_Lusatravel.xlsx
+++ b/docs/Guia_Documentacao_Viagem_Lusatravel.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -663,94 +663,108 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>• ASTERISCO (*) antes do nome do país na aba 'Por país' = destino com pelo menos uma informação incompleta ou a confirmar (em qualquer coluna, não só no Status). Revisar antes de orientar o cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>• Aba 'Outros documentos obrigatórios' reúne exigências que não dependem do destino: menores de idade, seguro viagem, comprovantes de entrada, formulários digitais, trânsito/conexão, e-DBV.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Fontes principais</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Embaixada da China no Brasil; Embaixada do Japão no Brasil; Home Office (Reino Unido); Comissão Europeia / EEAS (ETIAS/EES); SRE México; Anvisa; Detran-SP; Embaixada do Brasil em Bogotá (febre amarela/Colômbia); Copa Airlines (Panamá); CNJ / e-Notariado (AEV); AIMA Portugal; Receita Federal (e-DBV); Governo do Canadá (trânsito); portais oficiais de cartões de chegada (Check-Mig, e-Ticket, ED Card, DI Card, MDAC, eTravel, SGAC, IMUGA, D'Viajeros); Panrotas; CNN Brasil; mídia especializada em vistos (2026).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>Embaixada da China no Brasil; Embaixada do Japão no Brasil; Home Office (Reino Unido); Comissão Europeia / EEAS (ETIAS/EES); SRE México; Anvisa; Detran-SP; Embaixada do Brasil em Bogotá (febre amarela/Colômbia); Copa Airlines (Panamá); CNJ / e-Notariado (AEV); AIMA Portugal; Receita Federal (e-DBV); Governo do Canadá (trânsito); portais oficiais de cartões de chegada (Check-Mig, e-Ticket, ED Card, DI Card, MDAC, eTravel, SGAC, IMUGA, D'Viajeros); Panrotas; CNN Brasil; mídia especializada em vistos (2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>O site iatatravelcenter.com bloqueia acesso automatizado e não pôde ser consultado diretamente. O site da imigração da Austrália (immi.homeaffairs.gov.au) também não pôde ser consultado (lista TWOV).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>O que mudou na revisão 2 (19/09/2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>• Nova aba 'Outros documentos obrigatórios' (11 itens) — ver acima.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• 'Por país': 2 colunas novas — 'Formulário digital de entrada/saída' e 'Conexão / trânsito no país'.</t>
+          <t>• Nova aba 'Outros documentos obrigatórios' (11 itens) — ver acima.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• 'Por país': 9 destinos novos — Panamá, Costa Rica, Cuba, República Dominicana, Aruba, Curaçao, Singapura, Vietnã, Maldivas; Indonésia, Malásia e Filipinas separadas em linhas próprias (58 → 69 linhas).</t>
+          <t>• 'Por país': 2 colunas novas — 'Formulário digital de entrada/saída' e 'Conexão / trânsito no país'.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• Colômbia: Check-Mig obrigatório (entrada/saída/conexão) e CIVP de febre amarela não é mais exigido em voos do Brasil (Circular 018/2024).</t>
+          <t>• 'Por país': 9 destinos novos — Panamá, Costa Rica, Cuba, República Dominicana, Aruba, Curaçao, Singapura, Vietnã, Maldivas; Indonésia, Malásia e Filipinas separadas em linhas próprias (58 → 69 linhas).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• Panamá: febre amarela não é mais exigida. Turquia: passaporte válido por 150 dias. África do Sul: 2 páginas em branco. Egito: e-Visa US$ 30 (mar/2026).</t>
+          <t>• Colômbia: Check-Mig obrigatório (entrada/saída/conexão) e CIVP de febre amarela não é mais exigido em voos do Brasil (Circular 018/2024).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>• Espanha, Portugal e França: comprovantes de entrada (meios de subsistência, carta de invitación, termo de responsabilidade).</t>
+          <t>• Panamá: febre amarela não é mais exigida. Turquia: passaporte válido por 150 dias. África do Sul: 2 páginas em branco. Egito: e-Visa US$ 30 (mar/2026).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>• 'Autorizações eletrônicas': 16 linhas novas (Check-Mig, e-Ticket, ED Card, DI Card, eVisa/D'Viajeros Cuba, MDAC, eTravel, SGAC, e-VoA, IMUGA, e-Visa Vietnã/Índia/Egito, NZTD, JESTA).</t>
+          <t>• Espanha, Portugal e França: comprovantes de entrada (meios de subsistência, carta de invitación, termo de responsabilidade).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>• 'Autorizações eletrônicas': 16 linhas novas (Check-Mig, e-Ticket, ED Card, DI Card, eVisa/D'Viajeros Cuba, MDAC, eTravel, SGAC, e-VoA, IMUGA, e-Visa Vietnã/Índia/Egito, NZTD, JESTA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>• 'Vacinas e PID': emissão digital do CIVP, mudanças recentes de febre amarela, detalhe da AEV para menores, Covid-19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>• Asterisco (*) no nome dos destinos com informação incompleta em qualquer coluna.</t>
         </is>
       </c>
     </row>
@@ -858,7 +872,7 @@
       </c>
       <c r="B2" s="25" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>* Argentina</t>
         </is>
       </c>
       <c r="C2" s="24" t="inlineStr">
@@ -1126,7 +1140,7 @@
       </c>
       <c r="B6" s="25" t="inlineStr">
         <is>
-          <t>Bolívia</t>
+          <t>* Bolívia</t>
         </is>
       </c>
       <c r="C6" s="24" t="inlineStr">
@@ -1193,7 +1207,7 @@
       </c>
       <c r="B7" s="25" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>* Peru</t>
         </is>
       </c>
       <c r="C7" s="24" t="inlineStr">
@@ -1260,7 +1274,7 @@
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>Colômbia</t>
+          <t>* Colômbia</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
@@ -1327,7 +1341,7 @@
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>Equador</t>
+          <t>* Equador</t>
         </is>
       </c>
       <c r="C9" s="24" t="inlineStr">
@@ -1528,7 +1542,7 @@
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>* México</t>
         </is>
       </c>
       <c r="C12" s="24" t="inlineStr">
@@ -1595,7 +1609,7 @@
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>Panamá</t>
+          <t>* Panamá</t>
         </is>
       </c>
       <c r="C13" s="24" t="inlineStr">
@@ -1662,7 +1676,7 @@
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>* Costa Rica</t>
         </is>
       </c>
       <c r="C14" s="24" t="inlineStr">
@@ -1729,7 +1743,7 @@
       </c>
       <c r="B15" s="25" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>* Cuba</t>
         </is>
       </c>
       <c r="C15" s="24" t="inlineStr">
@@ -1796,7 +1810,7 @@
       </c>
       <c r="B16" s="25" t="inlineStr">
         <is>
-          <t>República Dominicana (Punta Cana)</t>
+          <t>* República Dominicana (Punta Cana)</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
@@ -1863,7 +1877,7 @@
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>Aruba</t>
+          <t>* Aruba</t>
         </is>
       </c>
       <c r="C17" s="24" t="inlineStr">
@@ -1926,7 +1940,7 @@
       </c>
       <c r="B18" s="25" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>* Curaçao</t>
         </is>
       </c>
       <c r="C18" s="24" t="inlineStr">
@@ -2525,7 +2539,7 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>Espanha</t>
+          <t>* Espanha</t>
         </is>
       </c>
       <c r="C27" s="24" t="inlineStr">
@@ -2927,7 +2941,7 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>Islândia</t>
+          <t>* Islândia</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
@@ -2994,7 +3008,7 @@
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>Itália</t>
+          <t>* Itália</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -3329,7 +3343,7 @@
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>Malta</t>
+          <t>* Malta</t>
         </is>
       </c>
       <c r="C39" s="24" t="inlineStr">
@@ -3932,7 +3946,7 @@
       </c>
       <c r="B48" s="25" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>* Reino Unido</t>
         </is>
       </c>
       <c r="C48" s="24" t="inlineStr">
@@ -4133,7 +4147,7 @@
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>Coreia do Sul</t>
+          <t>* Coreia do Sul</t>
         </is>
       </c>
       <c r="C51" s="24" t="inlineStr">
@@ -4200,7 +4214,7 @@
       </c>
       <c r="B52" s="25" t="inlineStr">
         <is>
-          <t>Tailândia</t>
+          <t>* Tailândia</t>
         </is>
       </c>
       <c r="C52" s="24" t="inlineStr">
@@ -4267,7 +4281,7 @@
       </c>
       <c r="B53" s="25" t="inlineStr">
         <is>
-          <t>Índia</t>
+          <t>* Índia</t>
         </is>
       </c>
       <c r="C53" s="24" t="inlineStr">
@@ -4330,7 +4344,7 @@
       </c>
       <c r="B54" s="25" t="inlineStr">
         <is>
-          <t>Indonésia</t>
+          <t>* Indonésia</t>
         </is>
       </c>
       <c r="C54" s="24" t="inlineStr">
@@ -4393,7 +4407,7 @@
       </c>
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>Malásia</t>
+          <t>* Malásia</t>
         </is>
       </c>
       <c r="C55" s="24" t="inlineStr">
@@ -4456,7 +4470,7 @@
       </c>
       <c r="B56" s="25" t="inlineStr">
         <is>
-          <t>Filipinas</t>
+          <t>* Filipinas</t>
         </is>
       </c>
       <c r="C56" s="24" t="inlineStr">
@@ -4519,7 +4533,7 @@
       </c>
       <c r="B57" s="25" t="inlineStr">
         <is>
-          <t>Singapura</t>
+          <t>* Singapura</t>
         </is>
       </c>
       <c r="C57" s="24" t="inlineStr">
@@ -4586,7 +4600,7 @@
       </c>
       <c r="B58" s="25" t="inlineStr">
         <is>
-          <t>Vietnã</t>
+          <t>* Vietnã</t>
         </is>
       </c>
       <c r="C58" s="24" t="inlineStr">
@@ -4653,7 +4667,7 @@
       </c>
       <c r="B59" s="25" t="inlineStr">
         <is>
-          <t>Maldivas</t>
+          <t>* Maldivas</t>
         </is>
       </c>
       <c r="C59" s="24" t="inlineStr">
@@ -4716,7 +4730,7 @@
       </c>
       <c r="B60" s="25" t="inlineStr">
         <is>
-          <t>Emirados Árabes Unidos</t>
+          <t>* Emirados Árabes Unidos</t>
         </is>
       </c>
       <c r="C60" s="24" t="inlineStr">
@@ -4779,7 +4793,7 @@
       </c>
       <c r="B61" s="25" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>* Israel</t>
         </is>
       </c>
       <c r="C61" s="24" t="inlineStr">
@@ -4846,7 +4860,7 @@
       </c>
       <c r="B62" s="25" t="inlineStr">
         <is>
-          <t>Turquia</t>
+          <t>* Turquia</t>
         </is>
       </c>
       <c r="C62" s="24" t="inlineStr">
@@ -4909,7 +4923,7 @@
       </c>
       <c r="B63" s="25" t="inlineStr">
         <is>
-          <t>Egito</t>
+          <t>* Egito</t>
         </is>
       </c>
       <c r="C63" s="24" t="inlineStr">
@@ -4972,7 +4986,7 @@
       </c>
       <c r="B64" s="25" t="inlineStr">
         <is>
-          <t>África do Sul</t>
+          <t>* África do Sul</t>
         </is>
       </c>
       <c r="C64" s="24" t="inlineStr">
@@ -5035,7 +5049,7 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>Marrocos</t>
+          <t>* Marrocos</t>
         </is>
       </c>
       <c r="C65" s="24" t="inlineStr">
@@ -5098,7 +5112,7 @@
       </c>
       <c r="B66" s="25" t="inlineStr">
         <is>
-          <t>Quênia</t>
+          <t>* Quênia</t>
         </is>
       </c>
       <c r="C66" s="24" t="inlineStr">
@@ -5161,7 +5175,7 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>Tanzânia</t>
+          <t>* Tanzânia</t>
         </is>
       </c>
       <c r="C67" s="24" t="inlineStr">
@@ -5224,7 +5238,7 @@
       </c>
       <c r="B68" s="25" t="inlineStr">
         <is>
-          <t>Austrália</t>
+          <t>* Austrália</t>
         </is>
       </c>
       <c r="C68" s="24" t="inlineStr">
@@ -5291,7 +5305,7 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>Nova Zelândia</t>
+          <t>* Nova Zelândia</t>
         </is>
       </c>
       <c r="C69" s="24" t="inlineStr">
@@ -5358,7 +5372,7 @@
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>Fiji</t>
+          <t>* Fiji</t>
         </is>
       </c>
       <c r="C70" s="24" t="inlineStr">

</xml_diff>